<commit_message>
deploy: main → 8377f68381ca5239aa793f29d601bb086052251d
</commit_message>
<xml_diff>
--- a/StructureDefinition-inera-ehds-allergy-intolerance.xlsx
+++ b/StructureDefinition-inera-ehds-allergy-intolerance.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-25T07:52:35+00:00</t>
+    <t>2026-09-30T09:02:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -629,7 +629,7 @@
     <t>abatement</t>
   </si>
   <si>
-    <t xml:space="preserve">Extension {allergyintolerance-abatement|5.3.0-ballot-tc1}
+    <t xml:space="preserve">Extension {allergyintolerance-abatement|5.3.0}
 </t>
   </si>
   <si>
@@ -639,7 +639,7 @@
     <t>The date or estimated date that the allergy or intolerance resolved. This is called abatement because of the many overloaded connotations associated with resolution.</t>
   </si>
   <si>
-    <t>Age is generally used when the patient reports an age at which the allergy or intolerance abated. If there is no abatement element, the clinicalStatus can be used to convey whether allergy or intolerance has resolved or not. When abatementString exists, it conveys that the allergy or intolerance is abated.</t>
+    <t>Age is generally used when the patient reports an age at which the AllergyIntolerance was abated. Period is generally used to convey an imprecise abatement date that occurred within the time period. Range is generally used to convey an imprecise age range (e.g. 4 to 6 years old). If there is no abatement element, the clinicalStatus can be used to convey whether allergy or intolerance has resolved or not. When abatementString exists, it conveys that the allergy or intolerance is abated.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1
@@ -693,7 +693,7 @@
     <t>AllergyIntolerance.clinicalStatus</t>
   </si>
   <si>
-    <t xml:space="preserve">CodeableConcept {http://hl7.org/fhir/uv/ips/StructureDefinition/CodeableConcept-uv-ips}
+    <t xml:space="preserve">CodeableConcept {http://hl7.org/fhir/uv/ips/StructureDefinition/CodeableConcept-uv-ips|2.0.1}
 </t>
   </si>
   <si>
@@ -865,7 +865,7 @@
     <t>Type of the substance/product, allergy or intolerance condition or a code for absent/unknown allergy.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/uv/ips/ValueSet/allergies-intolerances-uv-ips</t>
+    <t>http://hl7.org/fhir/uv/ips/ValueSet/allergies-intolerances-uv-ips|2.0.1</t>
   </si>
   <si>
     <t>substance/product:@@ -1233,7 +1233,7 @@
     <t>Code for the allergy or intolerance reaction manifestation from SNOMED CT.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/uv/ips/ValueSet/allergy-reaction-uv-ips</t>
+    <t>http://hl7.org/fhir/uv/ips/ValueSet/allergy-reaction-uv-ips|2.0.1</t>
   </si>
   <si>
     <t>AL1-5</t>
@@ -1648,7 +1648,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="71.2578125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="75.78515625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1663,7 +1663,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="106.67578125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="50.62109375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="54.4765625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>

</xml_diff>